<commit_message>
Update Work_Track.xlsx with latest data
</commit_message>
<xml_diff>
--- a/Work_Track.xlsx
+++ b/Work_Track.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dinesh_Academic\Projects\VS_Projects\ProfApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53A8FE3F-5096-4670-8B70-A3ECEDF42D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{607F2A01-FA41-495D-8A00-122EB9CDC28B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="602" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="602" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Academic" sheetId="2" r:id="rId1"/>
@@ -24,18 +24,31 @@
     <sheet name="Conferences" sheetId="4" r:id="rId9"/>
     <sheet name="Ideas" sheetId="5" r:id="rId10"/>
     <sheet name="History_record" sheetId="6" r:id="rId11"/>
+    <sheet name="Users" sheetId="14" r:id="rId12"/>
+    <sheet name="Contact" sheetId="16" r:id="rId13"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="500" uniqueCount="314">
   <si>
     <t>S. No.</t>
   </si>
@@ -547,9 +560,6 @@
     <t>Educational Details</t>
   </si>
   <si>
-    <t>Post-PhD</t>
-  </si>
-  <si>
     <t>Class X (AISSE)</t>
   </si>
   <si>
@@ -817,9 +827,6 @@
     <t>Sole Supervisor</t>
   </si>
   <si>
-    <t>Joint Supervsor</t>
-  </si>
-  <si>
     <t>Ramya Madhavaram</t>
   </si>
   <si>
@@ -890,13 +897,106 @@
   </si>
   <si>
     <t>Work Exp</t>
+  </si>
+  <si>
+    <t>Username</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>kdinesh</t>
+  </si>
+  <si>
+    <t>Kd94@profweb</t>
+  </si>
+  <si>
+    <t>Faculty</t>
+  </si>
+  <si>
+    <t>admin</t>
+  </si>
+  <si>
+    <t>admin123</t>
+  </si>
+  <si>
+    <t>Admin</t>
+  </si>
+  <si>
+    <t>K Dinesh</t>
+  </si>
+  <si>
+    <t>Prof. K Dinesh</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>profkdinesh@gmail.com</t>
+  </si>
+  <si>
+    <t>kdinesh@nitw.ac.in</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>91-870-2465038</t>
+  </si>
+  <si>
+    <t>Address Line 1</t>
+  </si>
+  <si>
+    <t>Address Line 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MS204, Department of Management Studies, </t>
+  </si>
+  <si>
+    <t>National Institute of Technology Warangal, Hanamkonda</t>
+  </si>
+  <si>
+    <t>Address Line 3</t>
+  </si>
+  <si>
+    <t>Telangana 506004, India</t>
+  </si>
+  <si>
+    <t>ORCID</t>
+  </si>
+  <si>
+    <t>Researchgate</t>
+  </si>
+  <si>
+    <t>LinkedIn</t>
+  </si>
+  <si>
+    <t>Scholar</t>
+  </si>
+  <si>
+    <t>https://scholar.google.com/citations?user=B9iz-gQAAAAJ&amp;hl=en&amp;oi=ao</t>
+  </si>
+  <si>
+    <t>https://www.scopus.com/authid/detail.uri?authorId=57210416499</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/kkdinesh/</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/profile/Kamala-Kannan-Dinesh</t>
+  </si>
+  <si>
+    <t>https://orcid.org/0000-0002-8956-8465</t>
+  </si>
+  <si>
+    <t>Joint Supervisor</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -924,6 +1024,28 @@
       <u/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1022,10 +1144,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1197,8 +1320,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="17" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="16">
@@ -1590,7 +1720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA8EC06E-E612-4927-AA85-EB849A64B331}">
-  <dimension ref="B4:G19"/>
+  <dimension ref="B4:G11"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="8.7265625" style="34"/>
@@ -1613,19 +1743,19 @@
         <v>0</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="F5" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="G5" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.35">
@@ -1633,10 +1763,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E6" s="38"/>
       <c r="F6" s="38">
@@ -1651,10 +1781,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="37" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="E7" s="38"/>
       <c r="F7" s="38">
@@ -1669,10 +1799,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D8" s="39" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="E8" s="38">
         <v>40784</v>
@@ -1689,10 +1819,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="E9" s="38">
         <v>42214</v>
@@ -1709,10 +1839,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E10" s="38">
         <v>43101</v>
@@ -1728,152 +1858,6 @@
       <c r="B11" s="35"/>
       <c r="C11" s="36"/>
       <c r="D11" s="36"/>
-    </row>
-    <row r="12" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="C12" s="33" t="s">
-        <v>170</v>
-      </c>
-      <c r="D12" s="33"/>
-    </row>
-    <row r="13" spans="2:7" s="36" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C13" s="40" t="s">
-        <v>167</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>175</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>172</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>173</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="14" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B14" s="14">
-        <v>1</v>
-      </c>
-      <c r="C14" s="37" t="s">
-        <v>218</v>
-      </c>
-      <c r="D14" s="37" t="s">
-        <v>182</v>
-      </c>
-      <c r="E14" s="38">
-        <v>44216</v>
-      </c>
-      <c r="F14" s="38">
-        <v>44742</v>
-      </c>
-      <c r="G14" s="46">
-        <v>20000</v>
-      </c>
-    </row>
-    <row r="15" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B15" s="14">
-        <v>2</v>
-      </c>
-      <c r="C15" s="37" t="s">
-        <v>168</v>
-      </c>
-      <c r="D15" s="37" t="s">
-        <v>182</v>
-      </c>
-      <c r="E15" s="38">
-        <v>44743</v>
-      </c>
-      <c r="F15" s="38">
-        <v>44926</v>
-      </c>
-      <c r="G15" s="46">
-        <v>75000</v>
-      </c>
-    </row>
-    <row r="16" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B16" s="14">
-        <v>3</v>
-      </c>
-      <c r="C16" s="37" t="s">
-        <v>183</v>
-      </c>
-      <c r="D16" s="37" t="s">
-        <v>182</v>
-      </c>
-      <c r="E16" s="38">
-        <v>45057</v>
-      </c>
-      <c r="F16" s="38">
-        <v>45169</v>
-      </c>
-      <c r="G16" s="46">
-        <v>45000</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B17" s="14">
-        <v>4</v>
-      </c>
-      <c r="C17" s="37" t="s">
-        <v>184</v>
-      </c>
-      <c r="D17" s="37" t="s">
-        <v>182</v>
-      </c>
-      <c r="E17" s="38">
-        <v>45200</v>
-      </c>
-      <c r="F17" s="38">
-        <v>45291</v>
-      </c>
-      <c r="G17" s="46">
-        <v>40000</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B18" s="14">
-        <v>5</v>
-      </c>
-      <c r="C18" s="37" t="s">
-        <v>185</v>
-      </c>
-      <c r="D18" s="37" t="s">
-        <v>186</v>
-      </c>
-      <c r="E18" s="38">
-        <v>45306</v>
-      </c>
-      <c r="F18" s="38">
-        <v>45869</v>
-      </c>
-      <c r="G18" s="46">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" x14ac:dyDescent="0.35">
-      <c r="B19" s="14">
-        <v>6</v>
-      </c>
-      <c r="C19" s="37" t="s">
-        <v>188</v>
-      </c>
-      <c r="D19" s="37" t="s">
-        <v>189</v>
-      </c>
-      <c r="E19" s="38">
-        <v>45880</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>190</v>
-      </c>
-      <c r="G19" s="14">
-        <v>111188</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3180,6 +3164,183 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8579A3B9-8840-4D67-962F-C12796B92DAF}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.54296875" customWidth="1"/>
+    <col min="2" max="2" width="14.6328125" customWidth="1"/>
+    <col min="3" max="3" width="16.90625" customWidth="1"/>
+    <col min="4" max="4" width="25.1796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="61" t="s">
+        <v>283</v>
+      </c>
+      <c r="B1" s="61" t="s">
+        <v>284</v>
+      </c>
+      <c r="C1" s="61" t="s">
+        <v>226</v>
+      </c>
+      <c r="D1" s="61" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>288</v>
+      </c>
+      <c r="B2" t="s">
+        <v>289</v>
+      </c>
+      <c r="C2" t="s">
+        <v>290</v>
+      </c>
+      <c r="D2" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3" s="60" t="s">
+        <v>286</v>
+      </c>
+      <c r="C3" t="s">
+        <v>287</v>
+      </c>
+      <c r="D3" t="s">
+        <v>292</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{9470CB24-902A-4DBE-8B51-E9B1D5226B81}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D8F7EA8-A9B3-473F-9D94-C86B5032E46B}">
+  <dimension ref="A2:C13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="13.1796875" style="61" customWidth="1"/>
+    <col min="2" max="2" width="22.26953125" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="61" t="s">
+        <v>250</v>
+      </c>
+      <c r="B2" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="61" t="s">
+        <v>293</v>
+      </c>
+      <c r="B3" s="60" t="s">
+        <v>294</v>
+      </c>
+      <c r="C3" s="60" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="61" t="s">
+        <v>296</v>
+      </c>
+      <c r="B4" s="62" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="61" t="s">
+        <v>298</v>
+      </c>
+      <c r="B5" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="61" t="s">
+        <v>299</v>
+      </c>
+      <c r="B6" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="61" t="s">
+        <v>302</v>
+      </c>
+      <c r="B7" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="61" t="s">
+        <v>304</v>
+      </c>
+      <c r="B9" s="60" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="61" t="s">
+        <v>305</v>
+      </c>
+      <c r="B10" s="60" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="61" t="s">
+        <v>306</v>
+      </c>
+      <c r="B11" s="60" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="61" t="s">
+        <v>307</v>
+      </c>
+      <c r="B12" s="60" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="61" t="s">
+        <v>37</v>
+      </c>
+      <c r="B13" s="60" t="s">
+        <v>309</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="6" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="B3" r:id="rId1" xr:uid="{10DFF167-F68C-4831-879F-2817F10C46FE}"/>
+    <hyperlink ref="C3" r:id="rId2" xr:uid="{F8268063-69CD-4631-B928-A6F6A3600B9F}"/>
+    <hyperlink ref="B12" r:id="rId3" xr:uid="{308E875D-E083-4C7F-8E8E-0DF25269D594}"/>
+    <hyperlink ref="B13" r:id="rId4" xr:uid="{0CAA5FE7-1CA4-4AFA-8E29-1D6515FEFE9B}"/>
+    <hyperlink ref="B11" r:id="rId5" xr:uid="{5A5E9386-0859-4D0B-88DA-A9B48EA02D91}"/>
+    <hyperlink ref="B10" r:id="rId6" xr:uid="{40FDD64F-7811-453B-BC7A-CBCE093E8AD2}"/>
+    <hyperlink ref="B9" r:id="rId7" xr:uid="{11A2C580-3E56-4CCD-B81C-8F282A48961B}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B0D01FD-168F-4E05-9976-928259C73ACA}">
   <dimension ref="B4:G11"/>
@@ -3196,7 +3357,7 @@
   <sheetData>
     <row r="4" spans="2:7" x14ac:dyDescent="0.35">
       <c r="C4" s="33" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="D4" s="33"/>
     </row>
@@ -3208,13 +3369,13 @@
         <v>167</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="E5" s="2" t="s">
+        <v>171</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>172</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>173</v>
       </c>
       <c r="G5" s="2" t="s">
         <v>7</v>
@@ -3225,10 +3386,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="37" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D6" s="37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E6" s="38">
         <v>44216</v>
@@ -3248,7 +3409,7 @@
         <v>168</v>
       </c>
       <c r="D7" s="37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E7" s="38">
         <v>44743</v>
@@ -3265,10 +3426,10 @@
         <v>3</v>
       </c>
       <c r="C8" s="37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D8" s="37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E8" s="38">
         <v>45057</v>
@@ -3285,10 +3446,10 @@
         <v>4</v>
       </c>
       <c r="C9" s="37" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D9" s="37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E9" s="38">
         <v>45200</v>
@@ -3305,10 +3466,10 @@
         <v>5</v>
       </c>
       <c r="C10" s="37" t="s">
+        <v>184</v>
+      </c>
+      <c r="D10" s="37" t="s">
         <v>185</v>
-      </c>
-      <c r="D10" s="37" t="s">
-        <v>186</v>
       </c>
       <c r="E10" s="38">
         <v>45306</v>
@@ -3325,16 +3486,16 @@
         <v>6</v>
       </c>
       <c r="C11" s="37" t="s">
+        <v>187</v>
+      </c>
+      <c r="D11" s="37" t="s">
         <v>188</v>
-      </c>
-      <c r="D11" s="37" t="s">
-        <v>189</v>
       </c>
       <c r="E11" s="38">
         <v>45880</v>
       </c>
       <c r="F11" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="G11" s="14">
         <v>111188</v>
@@ -3359,7 +3520,7 @@
   <sheetData>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="B2" s="36" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="36" customFormat="1" x14ac:dyDescent="0.35">
@@ -3367,16 +3528,16 @@
         <v>0</v>
       </c>
       <c r="B3" s="40" t="s">
+        <v>191</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>192</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>194</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
@@ -3384,60 +3545,68 @@
         <v>1</v>
       </c>
       <c r="B4" s="37" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="14" t="s">
         <v>196</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>197</v>
       </c>
       <c r="D4" s="17">
         <v>45883</v>
       </c>
-      <c r="E4" s="14"/>
+      <c r="E4" s="14" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="14">
         <v>2</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D5" s="17">
         <v>45883</v>
       </c>
-      <c r="E5" s="14"/>
+      <c r="E5" s="14" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="14">
         <v>3</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D6" s="17">
         <v>45883</v>
       </c>
-      <c r="E6" s="14"/>
+      <c r="E6" s="14" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="14">
         <v>4</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D7" s="17">
         <v>45883</v>
       </c>
-      <c r="E7" s="14"/>
+      <c r="E7" s="59">
+        <v>46204</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="14">
@@ -3482,34 +3651,34 @@
         <v>0</v>
       </c>
       <c r="B3" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>251</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>252</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="E3" s="7" t="s">
         <v>32</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="G3" s="28" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="H3" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="I3" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="J3" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="K3" s="2" t="s">
         <v>255</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>256</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>7</v>
@@ -3520,15 +3689,15 @@
         <v>1</v>
       </c>
       <c r="B4" s="45" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="C4" s="45"/>
       <c r="D4" s="14" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E4" s="45"/>
       <c r="F4" s="14" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="45"/>
@@ -3542,18 +3711,18 @@
         <v>2</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C5" s="45"/>
       <c r="D5" s="14" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="E5" s="45"/>
       <c r="F5" s="14" t="s">
-        <v>260</v>
+        <v>313</v>
       </c>
       <c r="G5" s="14" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="H5" s="45"/>
       <c r="I5" s="45"/>
@@ -4592,13 +4761,13 @@
       <c r="B4" s="16"/>
       <c r="C4" s="15"/>
       <c r="D4" s="16" t="s">
+        <v>200</v>
+      </c>
+      <c r="E4" s="16" t="s">
         <v>201</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="F4" s="16" t="s">
         <v>202</v>
-      </c>
-      <c r="F4" s="16" t="s">
-        <v>203</v>
       </c>
       <c r="G4" s="14" t="s">
         <v>10</v>
@@ -4754,7 +4923,7 @@
         <v>67</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G10" s="14" t="s">
         <v>10</v>
@@ -4777,10 +4946,10 @@
         <v>8</v>
       </c>
       <c r="E11" s="15" t="s">
+        <v>212</v>
+      </c>
+      <c r="F11" s="16" t="s">
         <v>213</v>
-      </c>
-      <c r="F11" s="16" t="s">
-        <v>214</v>
       </c>
       <c r="G11" s="14" t="s">
         <v>54</v>
@@ -4800,13 +4969,13 @@
       <c r="B12" s="16"/>
       <c r="C12" s="15"/>
       <c r="D12" s="16" t="s">
+        <v>243</v>
+      </c>
+      <c r="E12" s="16" t="s">
         <v>244</v>
       </c>
-      <c r="E12" s="16" t="s">
-        <v>245</v>
-      </c>
       <c r="F12" s="16" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G12" s="14" t="s">
         <v>10</v>
@@ -4826,13 +4995,13 @@
       <c r="B13" s="16"/>
       <c r="C13" s="15"/>
       <c r="D13" s="16" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="G13" s="14" t="s">
         <v>18</v>
@@ -4844,7 +5013,7 @@
         <v>46059</v>
       </c>
       <c r="J13" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
@@ -4940,7 +5109,7 @@
         <v>149</v>
       </c>
       <c r="F18" s="16" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G18" s="14" t="s">
         <v>10</v>
@@ -4960,13 +5129,13 @@
       <c r="B19" s="16"/>
       <c r="C19" s="15"/>
       <c r="D19" s="16" t="s">
+        <v>214</v>
+      </c>
+      <c r="E19" s="15" t="s">
         <v>215</v>
       </c>
-      <c r="E19" s="15" t="s">
+      <c r="F19" s="16" t="s">
         <v>216</v>
-      </c>
-      <c r="F19" s="16" t="s">
-        <v>217</v>
       </c>
       <c r="G19" s="14" t="s">
         <v>10</v>
@@ -4978,7 +5147,7 @@
         <v>45989</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
@@ -5108,19 +5277,19 @@
         <v>4</v>
       </c>
       <c r="B28" s="16" t="s">
+        <v>209</v>
+      </c>
+      <c r="C28" s="16" t="s">
+        <v>208</v>
+      </c>
+      <c r="D28" s="16" t="s">
+        <v>207</v>
+      </c>
+      <c r="E28" s="16" t="s">
+        <v>211</v>
+      </c>
+      <c r="F28" s="16" t="s">
         <v>210</v>
-      </c>
-      <c r="C28" s="16" t="s">
-        <v>209</v>
-      </c>
-      <c r="D28" s="16" t="s">
-        <v>208</v>
-      </c>
-      <c r="E28" s="16" t="s">
-        <v>212</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>211</v>
       </c>
       <c r="G28" s="14" t="s">
         <v>18</v>
@@ -5132,7 +5301,7 @@
         <v>45960</v>
       </c>
       <c r="J28" s="15" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
@@ -5587,7 +5756,7 @@
         <v>34</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="K2" s="28" t="s">
         <v>7</v>
@@ -5616,7 +5785,7 @@
         <v>36</v>
       </c>
       <c r="H3" s="27" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="I3" s="27" t="s">
         <v>144</v>
@@ -5625,7 +5794,7 @@
         <v>54</v>
       </c>
       <c r="K3" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="62" x14ac:dyDescent="0.35">
@@ -5651,16 +5820,16 @@
         <v>36</v>
       </c>
       <c r="H4" s="27" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="I4" s="27" t="s">
         <v>40</v>
       </c>
       <c r="J4" s="27" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K4" s="20" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="77.5" x14ac:dyDescent="0.35">
@@ -5692,10 +5861,10 @@
         <v>46</v>
       </c>
       <c r="J5" s="27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K5" s="20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="77.5" x14ac:dyDescent="0.35">
@@ -5727,7 +5896,7 @@
         <v>53</v>
       </c>
       <c r="J6" s="27" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K6" s="20"/>
     </row>
@@ -5760,7 +5929,7 @@
         <v>51</v>
       </c>
       <c r="J7" s="27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K7" s="20"/>
     </row>
@@ -5793,7 +5962,7 @@
         <v>66</v>
       </c>
       <c r="J8" s="27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K8" s="20"/>
     </row>
@@ -5826,7 +5995,7 @@
         <v>71</v>
       </c>
       <c r="J9" s="27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K9" s="20"/>
     </row>
@@ -5859,7 +6028,7 @@
         <v>77</v>
       </c>
       <c r="J10" s="27" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K10" s="20"/>
     </row>
@@ -5892,7 +6061,7 @@
         <v>81</v>
       </c>
       <c r="J11" s="27" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="K11" s="20"/>
     </row>
@@ -5925,7 +6094,7 @@
         <v>86</v>
       </c>
       <c r="J12" s="27" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="K12" s="20"/>
     </row>
@@ -6961,31 +7130,31 @@
   <sheetData>
     <row r="2" spans="1:10" s="1" customFormat="1" ht="31" x14ac:dyDescent="0.35">
       <c r="A2" s="28" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B2" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="E2" s="7" t="s">
         <v>219</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="E2" s="7" t="s">
+      <c r="F2" s="3" t="s">
         <v>220</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="28" t="s">
+        <v>240</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>222</v>
+      </c>
+      <c r="I2" s="2" t="s">
         <v>221</v>
-      </c>
-      <c r="G2" s="28" t="s">
-        <v>241</v>
-      </c>
-      <c r="H2" s="2" t="s">
-        <v>223</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>222</v>
       </c>
       <c r="J2" s="28" t="s">
         <v>7</v>
@@ -6996,19 +7165,19 @@
         <v>1</v>
       </c>
       <c r="B3" s="50" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="E3" s="53" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="F3" s="53" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G3" s="50">
         <v>48</v>
@@ -7017,7 +7186,7 @@
         <v>54</v>
       </c>
       <c r="I3" s="47" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="J3" s="50"/>
     </row>
@@ -7025,10 +7194,10 @@
       <c r="A4" s="58"/>
       <c r="B4" s="52"/>
       <c r="C4" s="43" t="s">
+        <v>229</v>
+      </c>
+      <c r="D4" s="42" t="s">
         <v>230</v>
-      </c>
-      <c r="D4" s="42" t="s">
-        <v>231</v>
       </c>
       <c r="E4" s="55"/>
       <c r="F4" s="55"/>
@@ -7042,19 +7211,19 @@
         <v>2</v>
       </c>
       <c r="B5" s="50" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C5" s="43" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E5" s="53" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="F5" s="53" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G5" s="50">
         <v>24</v>
@@ -7063,7 +7232,7 @@
         <v>45967</v>
       </c>
       <c r="I5" s="47" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="J5" s="50"/>
     </row>
@@ -7071,10 +7240,10 @@
       <c r="A6" s="57"/>
       <c r="B6" s="51"/>
       <c r="C6" s="16" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E6" s="54"/>
       <c r="F6" s="54"/>
@@ -7087,10 +7256,10 @@
       <c r="A7" s="57"/>
       <c r="B7" s="51"/>
       <c r="C7" s="16" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D7" s="16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E7" s="54"/>
       <c r="F7" s="54"/>
@@ -7103,10 +7272,10 @@
       <c r="A8" s="58"/>
       <c r="B8" s="52"/>
       <c r="C8" s="16" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E8" s="55"/>
       <c r="F8" s="55"/>
@@ -7120,19 +7289,19 @@
         <v>3</v>
       </c>
       <c r="B9" s="50" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C9" s="43" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D9" s="41" t="s">
+        <v>276</v>
+      </c>
+      <c r="E9" s="50" t="s">
         <v>278</v>
       </c>
-      <c r="E9" s="50" t="s">
-        <v>280</v>
-      </c>
       <c r="F9" s="50" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="G9" s="50">
         <v>12</v>
@@ -7141,7 +7310,7 @@
         <v>46157</v>
       </c>
       <c r="I9" s="47" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="J9" s="50"/>
     </row>
@@ -7149,10 +7318,10 @@
       <c r="A10" s="57"/>
       <c r="B10" s="51"/>
       <c r="C10" s="16" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E10" s="51"/>
       <c r="F10" s="51"/>
@@ -7165,10 +7334,10 @@
       <c r="A11" s="57"/>
       <c r="B11" s="51"/>
       <c r="C11" s="16" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E11" s="51"/>
       <c r="F11" s="51"/>
@@ -7181,10 +7350,10 @@
       <c r="A12" s="57"/>
       <c r="B12" s="51"/>
       <c r="C12" s="16" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="E12" s="51"/>
       <c r="F12" s="51"/>
@@ -7197,10 +7366,10 @@
       <c r="A13" s="58"/>
       <c r="B13" s="52"/>
       <c r="C13" s="16" t="s">
+        <v>275</v>
+      </c>
+      <c r="D13" s="16" t="s">
         <v>277</v>
-      </c>
-      <c r="D13" s="16" t="s">
-        <v>279</v>
       </c>
       <c r="E13" s="52"/>
       <c r="F13" s="52"/>

</xml_diff>